<commit_message>
Update Supabase integration by renaming environment variables for clarity and consistency. Modify related client and middleware functions to utilize new variable names. Adjust example environment file to reflect these changes. Additionally, update CSV templates to include new columns and improve structure for better usability.
</commit_message>
<xml_diff>
--- a/writing-task2-templates.xlsx
+++ b/writing-task2-templates.xlsx
@@ -815,10 +815,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="14" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1440,7 +1439,6 @@
       <c r="H5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="2"/>
       <c r="J5" t="s">
         <v>12</v>
       </c>
@@ -1504,212 +1502,212 @@
         <v>95</v>
       </c>
     </row>
-    <row r="7" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="H7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="I7" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="J7" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K7" s="3" t="s">
+      <c r="K7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="L7" s="3" t="s">
+      <c r="L7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="M7" s="3" t="s">
+      <c r="M7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="N7" s="3" t="s">
+      <c r="N7" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="O7" s="3" t="s">
+      <c r="O7" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="I8" s="4"/>
-      <c r="J8" s="3" t="s">
+      <c r="I8" s="3"/>
+      <c r="J8" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="K8" s="3" t="s">
+      <c r="K8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="L8" s="3" t="s">
+      <c r="L8" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="M8" s="3" t="s">
+      <c r="M8" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="N8" s="3" t="s">
+      <c r="N8" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="O8" s="3" t="s">
+      <c r="O8" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="P8" s="3" t="s">
+      <c r="P8" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="Q8" s="3" t="s">
+      <c r="Q8" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="R8" s="3" t="s">
+      <c r="R8" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="H9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="I9" s="4"/>
-      <c r="J9" s="3" t="s">
+      <c r="I9" s="3"/>
+      <c r="J9" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="K9" s="3" t="s">
+      <c r="K9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="L9" s="3" t="s">
+      <c r="L9" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="M9" s="3" t="s">
+      <c r="M9" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="N9" s="3" t="s">
+      <c r="N9" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="O9" s="3" t="s">
+      <c r="O9" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="P9" s="3" t="s">
+      <c r="P9" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="Q9" s="3" t="s">
+      <c r="Q9" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="R9" s="3" t="s">
+      <c r="R9" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="10" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
+    <row r="10" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="H10" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="I10" s="4"/>
-      <c r="J10" s="3" t="s">
+      <c r="I10" s="3"/>
+      <c r="J10" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="K10" s="3" t="s">
+      <c r="K10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="L10" s="3" t="s">
+      <c r="L10" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="M10" s="3" t="s">
+      <c r="M10" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="N10" s="3" t="s">
+      <c r="N10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="O10" s="3" t="s">
+      <c r="O10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="P10" s="3" t="s">
+      <c r="P10" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="Q10" s="3" t="s">
+      <c r="Q10" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="R10" s="3" t="s">
+      <c r="R10" s="2" t="s">
         <v>79</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add deduplication functionality for task2 templates
Implement dedupeRowsByText function to merge sentence rows with identical text, consolidating type IDs for shared sentences. Update HomePage and test suite to utilize this new functionality, ensuring consistent handling of background sentences across essay types. Enhance test coverage for deduplication scenarios.
</commit_message>
<xml_diff>
--- a/writing-task2-templates.xlsx
+++ b/writing-task2-templates.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\skvop\Project\_new\ielts-tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{399CF8D4-669D-48BF-96DB-3390775F7E5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B098E03A-FF7C-4C64-8392-AFD8E8A6E7D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{BBF97831-2D31-40A8-9089-F1CEFA2DC268}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{BBF97831-2D31-40A8-9089-F1CEFA2DC268}"/>
   </bookViews>
   <sheets>
     <sheet name="writing-task2-templates" sheetId="1" r:id="rId1"/>
+    <sheet name="工作表1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="123">
   <si>
     <t>文章類型</t>
   </si>
@@ -308,6 +309,87 @@
   </si>
   <si>
     <t>In conclusion, M1; however, M2. Personally, I believe Op.</t>
+  </si>
+  <si>
+    <t>B1-6</t>
+  </si>
+  <si>
+    <t>B2-6</t>
+  </si>
+  <si>
+    <t>This phenomenon could bring about A1 and A2, but it could also lead to D1 and D2.</t>
+  </si>
+  <si>
+    <t>This essay will discuss both of these aspects in detail.</t>
+  </si>
+  <si>
+    <t>One main benefit is that A1.</t>
+  </si>
+  <si>
+    <t>Apart from that, another benefit is that A2.</t>
+  </si>
+  <si>
+    <t>However, one main drawback is that D1.</t>
+  </si>
+  <si>
+    <t>Moreover, another drawback is that D2.</t>
+  </si>
+  <si>
+    <t>In conclusion, although this phenomenon can bring about A1 and A2, it can also lead to D1 and D2.</t>
+  </si>
+  <si>
+    <t>In modern society, T has become a pressing issue.</t>
+  </si>
+  <si>
+    <t>This phenomenon could bring about P1 and P2, but these problems can be alleviated by S1 and S2.</t>
+  </si>
+  <si>
+    <t>One main problem is that P1.</t>
+  </si>
+  <si>
+    <t>Apart from that, another problem is that P2.</t>
+  </si>
+  <si>
+    <t>To alleviate these problems, one main solution is that S1.</t>
+  </si>
+  <si>
+    <t>Moreover, another solution is that S2.</t>
+  </si>
+  <si>
+    <t>In conclusion, although this phenomenon can bring about P1 and P2, these problems can be alleviated by S1 and S2.</t>
+  </si>
+  <si>
+    <t>This phenomenon could be attributed to C1 and C2, but it can be alleviated by S1 and S2.</t>
+  </si>
+  <si>
+    <t>One main cause is that C1.</t>
+  </si>
+  <si>
+    <t>Apart from that, another cause is that C2.</t>
+  </si>
+  <si>
+    <t>To alleviate this problem, one main solution is that S1.</t>
+  </si>
+  <si>
+    <t>In conclusion, although this phenomenon can be attributed to C1 and C2, it can be alleviated by S1 and S2.</t>
+  </si>
+  <si>
+    <t>This phenomenon could be attributed to C1 and C2, and it could lead to Ef1 and Ef2.</t>
+  </si>
+  <si>
+    <t>As for the effects, one main impact is that Ef1.</t>
+  </si>
+  <si>
+    <t>Moreover, another impact is that Ef2.</t>
+  </si>
+  <si>
+    <t>In conclusion, this phenomenon can be attributed to C1 and C2, and it can lead to Ef1 and Ef2.</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>x`</t>
   </si>
 </sst>
 </file>
@@ -1716,4 +1798,563 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39510D22-2F5F-447F-8329-FD2ED5A0C9EA}">
+  <dimension ref="A1:Q10"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="36.8984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="55.296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="80.69921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="90" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="34" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.09765625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.09765625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="40.796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.59765625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="47.09765625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.59765625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.09765625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.59765625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="40.796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.59765625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="95.296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E1" t="s">
+        <v>84</v>
+      </c>
+      <c r="F1" t="s">
+        <v>85</v>
+      </c>
+      <c r="G1" t="s">
+        <v>86</v>
+      </c>
+      <c r="H1" t="s">
+        <v>87</v>
+      </c>
+      <c r="I1" t="s">
+        <v>88</v>
+      </c>
+      <c r="J1" t="s">
+        <v>96</v>
+      </c>
+      <c r="K1" t="s">
+        <v>89</v>
+      </c>
+      <c r="L1" t="s">
+        <v>90</v>
+      </c>
+      <c r="M1" t="s">
+        <v>91</v>
+      </c>
+      <c r="N1" t="s">
+        <v>92</v>
+      </c>
+      <c r="O1" t="s">
+        <v>93</v>
+      </c>
+      <c r="P1" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="K2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="K3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="K4" t="s">
+        <v>28</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="K5" t="s">
+        <v>12</v>
+      </c>
+      <c r="L5" t="s">
+        <v>13</v>
+      </c>
+      <c r="M5" t="s">
+        <v>14</v>
+      </c>
+      <c r="N5" t="s">
+        <v>15</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I6" t="s">
+        <v>35</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="K6" t="s">
+        <v>36</v>
+      </c>
+      <c r="L6" t="s">
+        <v>13</v>
+      </c>
+      <c r="M6" t="s">
+        <v>14</v>
+      </c>
+      <c r="N6" t="s">
+        <v>15</v>
+      </c>
+      <c r="O6" t="s">
+        <v>37</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D7" t="s">
+        <v>99</v>
+      </c>
+      <c r="E7" t="s">
+        <v>100</v>
+      </c>
+      <c r="F7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" t="s">
+        <v>9</v>
+      </c>
+      <c r="H7" t="s">
+        <v>10</v>
+      </c>
+      <c r="I7" t="s">
+        <v>101</v>
+      </c>
+      <c r="J7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K7" t="s">
+        <v>102</v>
+      </c>
+      <c r="L7" t="s">
+        <v>44</v>
+      </c>
+      <c r="M7" t="s">
+        <v>14</v>
+      </c>
+      <c r="N7" t="s">
+        <v>15</v>
+      </c>
+      <c r="O7" t="s">
+        <v>103</v>
+      </c>
+      <c r="P7" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C8" t="s">
+        <v>106</v>
+      </c>
+      <c r="D8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E8" t="s">
+        <v>107</v>
+      </c>
+      <c r="F8" t="s">
+        <v>8</v>
+      </c>
+      <c r="G8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H8" t="s">
+        <v>10</v>
+      </c>
+      <c r="I8" t="s">
+        <v>108</v>
+      </c>
+      <c r="J8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K8" t="s">
+        <v>109</v>
+      </c>
+      <c r="L8" t="s">
+        <v>44</v>
+      </c>
+      <c r="M8" t="s">
+        <v>14</v>
+      </c>
+      <c r="N8" t="s">
+        <v>15</v>
+      </c>
+      <c r="O8" t="s">
+        <v>110</v>
+      </c>
+      <c r="P8" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" t="s">
+        <v>105</v>
+      </c>
+      <c r="C9" t="s">
+        <v>112</v>
+      </c>
+      <c r="D9" t="s">
+        <v>99</v>
+      </c>
+      <c r="E9" t="s">
+        <v>113</v>
+      </c>
+      <c r="F9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" t="s">
+        <v>9</v>
+      </c>
+      <c r="H9" t="s">
+        <v>10</v>
+      </c>
+      <c r="I9" t="s">
+        <v>114</v>
+      </c>
+      <c r="J9" t="s">
+        <v>13</v>
+      </c>
+      <c r="K9" t="s">
+        <v>115</v>
+      </c>
+      <c r="L9" t="s">
+        <v>44</v>
+      </c>
+      <c r="M9" t="s">
+        <v>14</v>
+      </c>
+      <c r="N9" t="s">
+        <v>15</v>
+      </c>
+      <c r="O9" t="s">
+        <v>110</v>
+      </c>
+      <c r="P9" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" t="s">
+        <v>117</v>
+      </c>
+      <c r="D10" t="s">
+        <v>99</v>
+      </c>
+      <c r="E10" t="s">
+        <v>113</v>
+      </c>
+      <c r="F10" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10" t="s">
+        <v>9</v>
+      </c>
+      <c r="H10" t="s">
+        <v>10</v>
+      </c>
+      <c r="I10" t="s">
+        <v>114</v>
+      </c>
+      <c r="J10" t="s">
+        <v>13</v>
+      </c>
+      <c r="K10" t="s">
+        <v>118</v>
+      </c>
+      <c r="L10" t="s">
+        <v>44</v>
+      </c>
+      <c r="M10" t="s">
+        <v>14</v>
+      </c>
+      <c r="N10" t="s">
+        <v>15</v>
+      </c>
+      <c r="O10" t="s">
+        <v>119</v>
+      </c>
+      <c r="P10" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>120</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>